<commit_message>
feat: add Gap Analysis and Received From columns to master inventory
Updated BTRC_Master_Data_Inventory.xlsx (16 columns):
- Added Received From: operator/org that submitted each file
- Added Gap Analysis: colour-coded gap description per dataset
  (green=no gap, amber=partial gap, red=100% not implemented)
- Dates carried forward from user-reviewed Excel

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MapData/BTRC_Master_Data_Inventory.xlsx
+++ b/MapData/BTRC_Master_Data_Inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Data Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Data Inventory'!$A$4:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Data Inventory'!$A$4:$P$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Master Data Inventory'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,7 +71,22 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00166534"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="0092400E"/>
       <sz val="9"/>
     </font>
@@ -181,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -207,6 +222,9 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -216,22 +234,28 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -599,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -608,14 +632,16 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -628,12 +654,12 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per dataset. Combines: received file details, data type analysis, usage status, and remarks.</t>
+          <t>One row per dataset. Covers: received file details, source, data types, usage status, gap analysis, and remarks.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="4" customHeight="1"/>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>S/N</t>
@@ -666,40 +692,50 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Received From</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
           <t>Records / Features</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Geometry</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Sub-types / Categories</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Key Attributes</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Coord System</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Data Period</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Used on Map?</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Gap Analysis</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Notes / Remarks</t>
         </is>
@@ -712,7 +748,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="72" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>1</v>
       </c>
@@ -743,43 +779,53 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
+          <t>Grameenphone (GP)</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
           <t>23,864</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>Fiber Connected: 8,971
 MW (Microwave): 14,893</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>Site Code, Latitude, Longitude, TX Type (Fiber / MW)</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
-        <is>
-          <t>All sites on map. Admin (Division / District / Upazila) enriched via point-in-polygon lookup. 246 border-edge sites show '—' for admin.</t>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Admin (Division / District / Upazila) enriched via point-in-polygon lookup. 246 border-edge sites show '--' for admin fields.</t>
         </is>
       </c>
     </row>
@@ -790,7 +836,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="72" customHeight="1">
+    <row r="8" ht="80" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>2</v>
       </c>
@@ -821,44 +867,54 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
+          <t>Robi Axiata</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
           <t>18,838</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>MW Only: 13,760
 Fiber Only: 1,632
 MW + Fiber (Both): 3,446</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>Site Code, Latitude, Longitude, MW flag (Yes / –), Fiber flag (Yes / –)</t>
-        </is>
-      </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
+          <t>Site Code, Latitude, Longitude, MW flag (Yes / --), Fiber flag (Yes / --)</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>All sites on map. Three-category backhaul classification applied. Admin enriched via PIP. 169 border-edge sites show '—'.</t>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Three-category backhaul classification applied. Admin enriched via PIP. 169 border-edge sites show '--'.</t>
         </is>
       </c>
     </row>
@@ -869,7 +925,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="72" customHeight="1">
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>3</v>
       </c>
@@ -900,120 +956,140 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
+          <t>Banglalink</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
           <t>15,154</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>Microwave: 13,015
 Fiber: 2,113
 Inactive: 26</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>Unique Site ID, Lat, Lon, Division, District, Thana, Address, MW Link Status, Fiber Optic Status, Primary Backhaul Type</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>All sites on map. Admin data taken directly from Excel (no PIP needed). Address field included in popup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="9" t="n">
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>Admin data taken directly from Excel (no PIP needed). Address field included in popup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Banglalink</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>BTS Towers — Historical</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>3gtower.geojson</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Banglalink</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>13,208</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>4G sites
 3G only
 2G only</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>Site Code, Site Name, Generation (2G/3G/4G), Division, District, Upazila, Union, Vendor</t>
         </is>
       </c>
-      <c r="K11" s="11" t="inlineStr">
+      <c r="L11" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L11" s="11" t="inlineStr">
+      <c r="M11" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N11" s="11" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>Historical tower dataset. Filterable by generation on map.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="72" customHeight="1">
+    <row r="12" ht="80" customHeight="1">
       <c r="A12" s="5" t="n">
         <v>5</v>
       </c>
@@ -1044,42 +1120,52 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
+          <t>Banglalink</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
           <t>172</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>72 Core
 48 Core
 32 Core</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>Core Count</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
         <is>
           <t>Historical fiber route lines. Filterable by core count on map.</t>
         </is>
@@ -1092,7 +1178,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="72" customHeight="1">
+    <row r="14" ht="80" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>6</v>
       </c>
@@ -1123,15 +1209,20 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
+          <t>BTCL</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
           <t>24,142</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>CP (Connection Point)
 HH (Hand Hole)
@@ -1142,72 +1233,82 @@
 (3,432 raw type values normalised to 6 categories)</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>Name, Latitude, Longitude, Point Type, Raw Type, Year, Feature Code</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>24,073 on map (69 removed by PIP — coordinates outside Bangladesh boundary; likely data-entry errors near borders).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="72" customHeight="1">
-      <c r="A15" s="9" t="n">
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>69 records removed (0.3% of total). Coordinates fell outside Bangladesh boundary — likely data-entry errors.</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>24,073 of 24,142 on map. Filtered points near borders should be verified and resubmitted by BTCL with corrected coordinates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>Fiber Lines — Historical</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>btcl-nttn-line.geojson</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>BTCL</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>584</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>MultiLineString</t>
         </is>
       </c>
-      <c r="I15" s="11" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>144+ Core
 96 Core
@@ -1216,33 +1317,38 @@
 &lt;24 Core</t>
         </is>
       </c>
-      <c r="J15" s="11" t="inlineStr">
+      <c r="K15" s="12" t="inlineStr">
         <is>
           <t>Operator Name, Line Name, Line Type, Core Count, Route Length (km), Cable Length (km), Duct Info, Division / District / Upazila</t>
         </is>
       </c>
-      <c r="K15" s="11" t="inlineStr">
+      <c r="L15" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L15" s="11" t="inlineStr">
+      <c r="M15" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M15" s="8" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N15" s="11" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P15" s="12" t="inlineStr">
         <is>
           <t>All lines on map. Filterable by core-count band.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="72" customHeight="1">
+    <row r="16" ht="80" customHeight="1">
       <c r="A16" s="5" t="n">
         <v>8</v>
       </c>
@@ -1273,15 +1379,20 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
+          <t>BTCL</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
           <t>29,795</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>HOP
 HH (Hand Hole)
@@ -1289,97 +1400,112 @@
 MH (Man Hole)</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>Operator Name, Point Name, Point Type, Lat, Lon, Division, District, Upazila, Union, Mouza, Year</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N16" s="7" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
         <is>
           <t>All nodes on map. Filterable by node type.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="72" customHeight="1">
-      <c r="A17" s="9" t="n">
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Union Project Locations</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>btcl-union-project-location.geojson</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>BTCL</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
         <is>
           <t>966</t>
         </is>
       </c>
-      <c r="H17" s="11" t="inlineStr">
+      <c r="I17" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I17" s="11" t="inlineStr">
+      <c r="J17" s="12" t="inlineStr">
         <is>
           <t>Union-level project markers</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="K17" s="12" t="inlineStr">
         <is>
           <t>Location coordinates</t>
         </is>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="L17" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L17" s="11" t="inlineStr">
+      <c r="M17" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M17" s="8" t="inlineStr">
+      <c r="N17" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N17" s="11" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P17" s="12" t="inlineStr">
         <is>
           <t>All union project markers on map.</t>
         </is>
@@ -1392,7 +1518,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="72" customHeight="1">
+    <row r="19" ht="80" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>10</v>
       </c>
@@ -1424,88 +1550,105 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
+          <t>Fiber@Home / FHLFON</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
           <t>141,567</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>Aerial: 85,366
 Burial: 53,870
 OPGW: 2,331</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>Operator Code, Operator Name, Infra Type (Own / Leased), Line ID, Year, Month, Line Name, Line Type, Path Along, Duct No, Duct Use, Cable No</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="M19" s="12" t="inlineStr">
+      <c r="N19" s="14" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
-        <is>
-          <t>Only 18,405 of 141,567 lines currently on map (13%). Full re-ingestion from FHLFONLineExcel.xlsx needed. OPGW lines (2,331) also not yet shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="72" customHeight="1">
-      <c r="A20" s="9" t="n">
+      <c r="O19" s="15" t="inlineStr">
+        <is>
+          <t>123,162 lines not yet on map (87% gap).
+Currently showing: 18,405 of 141,567.
+Missing: full Aerial set (85k), full Burial set (53k), all OPGW (2,331).</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Full re-ingestion from FHLFONLineExcel.xlsx required. Current map uses only a pre-converted subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Fiber@Home (FHLFON)</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>FHLFONPoint.shp + FHLFONPointExcel.xlsx
 (10 files: 8 shapefile + 1 Excel + 1 duplicate)</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Shapefile + XLSX</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Fiber@Home / FHLFON</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>122,150</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="I20" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>JE (Joint Enclosure): 38,097
 EP (End Point): 25,804
@@ -1524,29 +1667,36 @@
 Other / Noise: ~44</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="K20" s="12" t="inlineStr">
         <is>
           <t>Year, Month, Operator Code, Operator Name, Point ID, Point Type, Point Name, Address, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="K20" s="11" t="inlineStr">
+      <c r="L20" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L20" s="11" t="inlineStr">
+      <c r="M20" s="12" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="M20" s="12" t="inlineStr">
+      <c r="N20" s="14" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="N20" s="11" t="inlineStr">
-        <is>
-          <t>94,953 of 122,150 on map (78%). Missing types: Coupler (22,435), FL (16,558), BDB (1,390), Pole (479), LDP (387), PIT (26), Customer (25). Note: 'Copy of FHLFONPointExcel.xlsx' is an exact duplicate — not used.</t>
+      <c r="O20" s="15" t="inlineStr">
+        <is>
+          <t>27,197 points not on map (22% gap).
+Currently showing: 94,953 of 122,150.
+Missing types: Coupler (22,435), FL (16,558), BDB (1,390), Pole (479), LDP (387), PIT (26), Customer (25).</t>
+        </is>
+      </c>
+      <c r="P20" s="12" t="inlineStr">
+        <is>
+          <t>'Copy of FHLFONPointExcel.xlsx' is an exact duplicate and not used.</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1707,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="72" customHeight="1">
+    <row r="22" ht="80" customHeight="1">
       <c r="A22" s="5" t="n">
         <v>12</v>
       </c>
@@ -1589,15 +1739,20 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
+          <t>Summit Communications</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
           <t>102,514</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>Aerial: 78,499
 Burial: 22,702
@@ -1606,73 +1761,85 @@
 Burial (Damaged): 89</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>FID, Line ID, Year, Month, Operator Code, Operator Name, Infra Type, Line Type, Line Name, Path Along, No of Ducts, Duct Use</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
+      <c r="L22" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L22" s="7" t="inlineStr">
+      <c r="M22" s="7" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="M22" s="12" t="inlineStr">
+      <c r="N22" s="14" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>Only 23,157 of 102,514 lines on map (23%). Full re-ingestion from Line_data.xlsx needed. Missing ~79,357 lines (mostly Aerial and Burial).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="72" customHeight="1">
-      <c r="A23" s="9" t="n">
+      <c r="O22" s="15" t="inlineStr">
+        <is>
+          <t>79,357 lines not on map (77% gap).
+Currently showing: 23,157 of 102,514.
+Missing: majority of Aerial (78k) and Burial (22k) lines.</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>Full re-ingestion from Line_data.xlsx required. Current map uses a simplified 3-tier classification only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Summit Communications</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Point_data.xlsx + Point_data.shp
 (1 Excel + multiple shapefile components)</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>XLSX + Shapefile</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Summit Communications</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>68,850</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="J23" s="12" t="inlineStr">
         <is>
           <t>TJB (Joint Box): 37,909
 HH (Hand Hole): 9,506
@@ -1691,33 +1858,40 @@
 Other: ~183</t>
         </is>
       </c>
-      <c r="J23" s="11" t="inlineStr">
+      <c r="K23" s="12" t="inlineStr">
         <is>
           <t>FID, Point ID, Year, Month, Operator Code, Operator Name, Point Type, Point Name, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
+      <c r="L23" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L23" s="11" t="inlineStr">
+      <c r="M23" s="12" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="M23" s="12" t="inlineStr">
+      <c r="N23" s="14" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="N23" s="11" t="inlineStr">
-        <is>
-          <t>14,562 of 68,850 on map (21%). Missing: TJB (37,909), EP (6,872), ODB (1,193), Node/TT (812), POP (666), POC (453), BS (422), Node/CBD (245), COLO/PoP (128), FAT (89), FDT (62) and others.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="72" customHeight="1">
+      <c r="O23" s="15" t="inlineStr">
+        <is>
+          <t>54,288 points not on map (79% gap).
+Currently showing: 14,562 of 68,850.
+Missing: TJB (37,909), EP (6,872), ODB (1,193), Node/TT (812), POP (666), POC (453), BS (422), Node/CBD (245), COLO/PoP (128), FAT (89), FDT (62).</t>
+        </is>
+      </c>
+      <c r="P23" s="12" t="inlineStr">
+        <is>
+          <t>Only Nodes (5,949) and BTS (8,613) currently on map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1">
       <c r="A24" s="5" t="n">
         <v>14</v>
       </c>
@@ -1748,42 +1922,52 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
+          <t>Summit Communications</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>Unknown — archive not extracted</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K24" s="7" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="L24" s="7" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="M24" s="13" t="inlineStr">
+      <c r="N24" s="16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N24" s="7" t="inlineStr">
-        <is>
-          <t>Archive file in Railway folder. Contents not yet extracted or analysed. May contain additional network data.</t>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>Not yet extracted. Content and size unknown.</t>
+        </is>
+      </c>
+      <c r="P24" s="7" t="inlineStr">
+        <is>
+          <t>Archive file found in Railway folder. Must be extracted and analysed to determine if it contains additional network data.</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1978,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="72" customHeight="1">
+    <row r="26" ht="80" customHeight="1">
       <c r="A26" s="5" t="n">
         <v>15</v>
       </c>
@@ -1826,112 +2010,132 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
+          <t>Bahon Limited</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
           <t>~7,763</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>Overhead (OH)
 Underground (UG)
 Wall Clamped (WC)</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>Cable Type, Division, District, Upazila (from DBF attributes)</t>
         </is>
       </c>
-      <c r="K26" s="7" t="inlineStr">
+      <c r="L26" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L26" s="7" t="inlineStr">
+      <c r="M26" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M26" s="8" t="inlineStr">
+      <c r="N26" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>All lines on map. Shapefile only — no Excel counterpart received. Exact record count unverified from DBF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="72" customHeight="1">
-      <c r="A27" s="9" t="n">
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>No significant gap detected. Exact source count unverified (shapefile only — no Excel counterpart for cross-check).</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>No Excel submission received from Bahon. Request Excel tabular data for BTRC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Bahon Limited</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>(Derived from shapefile dataset)</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Shapefile</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Bahon Limited</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>12,817</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>Network junction nodes</t>
         </is>
       </c>
-      <c r="J27" s="11" t="inlineStr">
+      <c r="K27" s="12" t="inlineStr">
         <is>
           <t>Node coordinates</t>
         </is>
       </c>
-      <c r="K27" s="11" t="inlineStr">
+      <c r="L27" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L27" s="11" t="inlineStr">
+      <c r="M27" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M27" s="8" t="inlineStr">
+      <c r="N27" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N27" s="11" t="inlineStr">
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -1944,7 +2148,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="72" customHeight="1">
+    <row r="29" ht="80" customHeight="1">
       <c r="A29" s="5" t="n">
         <v>17</v>
       </c>
@@ -1976,15 +2180,20 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
+          <t>InfoSarkar-3 / FHL</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
           <t>3,383</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>48 Core
 24 Core
@@ -1994,97 +2203,112 @@
 CBD</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>Core count, Name, Layer, Length (km)</t>
         </is>
       </c>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="L29" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="M29" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M29" s="8" t="inlineStr">
+      <c r="N29" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N29" s="7" t="inlineStr">
+      <c r="O29" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr">
         <is>
           <t>All lines on map with core-count filter.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="72" customHeight="1">
-      <c r="A30" s="9" t="n">
+    <row r="30" ht="80" customHeight="1">
+      <c r="A30" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>InfoSarkar-3 (IS3)</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>doc.kml (same file)</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>KML</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G30" s="11" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>InfoSarkar-3 / FHL</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
         <is>
           <t>477</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="I30" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I30" s="11" t="inlineStr">
+      <c r="J30" s="12" t="inlineStr">
         <is>
           <t>Network junction nodes</t>
         </is>
       </c>
-      <c r="J30" s="11" t="inlineStr">
+      <c r="K30" s="12" t="inlineStr">
         <is>
           <t>Node coordinates</t>
         </is>
       </c>
-      <c r="K30" s="11" t="inlineStr">
+      <c r="L30" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L30" s="11" t="inlineStr">
+      <c r="M30" s="12" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M30" s="8" t="inlineStr">
+      <c r="N30" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N30" s="11" t="inlineStr">
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P30" s="12" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -2097,7 +2321,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="72" customHeight="1">
+    <row r="32" ht="80" customHeight="1">
       <c r="A32" s="5" t="n">
         <v>19</v>
       </c>
@@ -2128,15 +2352,20 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
+          <t>PGCB</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
           <t>324</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>400 kV Transmission Line
 230 kV Transmission Line
@@ -2145,27 +2374,32 @@
 Others</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>Layer (voltage / type), Name, Description</t>
         </is>
       </c>
-      <c r="K32" s="7" t="inlineStr">
+      <c r="L32" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L32" s="7" t="inlineStr">
+      <c r="M32" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M32" s="8" t="inlineStr">
+      <c r="N32" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N32" s="7" t="inlineStr">
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>All OPGW lines on map. Filterable by voltage / line type.</t>
         </is>
@@ -2179,7 +2413,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="72" customHeight="1">
+    <row r="34" ht="80" customHeight="1">
       <c r="A34" s="5" t="n">
         <v>20</v>
       </c>
@@ -2211,113 +2445,143 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
+          <t>BTRC / Multiple Operators</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
           <t>8,163</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>By operator: Grameenphone, Robi, BTCL,
-Banglalink, MOTN, BSCCL, Unknown</t>
-        </is>
-      </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
+          <t>Grameenphone
+Robi
+BTCL
+Banglalink
+MOTN
+BSCCL
+Unknown</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
           <t>Name, Operator, Distance (km)</t>
         </is>
       </c>
-      <c r="K34" s="7" t="inlineStr">
+      <c r="L34" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L34" s="7" t="inlineStr">
+      <c r="M34" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M34" s="8" t="inlineStr">
+      <c r="N34" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N34" s="7" t="inlineStr">
-        <is>
-          <t>All 6-operator inter-district fiber lines on map. Operator colour filter applied.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="72" customHeight="1">
-      <c r="A35" s="9" t="n">
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P34" s="7" t="inlineStr">
+        <is>
+          <t>All 6-operator inter-district fiber lines on map with operator colour filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="80" customHeight="1">
+      <c r="A35" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Multi-operator
 (GP, Robi, BTCL, BL, MOTN, BSCCL)</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>Fiber Network — Points</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>fiber_network_multiple_district.kmz (same file)</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>KMZ</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>BTRC / Multiple Operators</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
         <is>
           <t>19,096</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="I35" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I35" s="11" t="inlineStr">
-        <is>
-          <t>By operator: Grameenphone, Robi, BTCL,
-Banglalink, MOTN, BSCCL, Unknown</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="inlineStr">
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>Grameenphone
+Robi
+BTCL
+Banglalink
+MOTN
+BSCCL
+Unknown</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
         <is>
           <t>Name, Operator</t>
         </is>
       </c>
-      <c r="K35" s="11" t="inlineStr">
+      <c r="L35" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L35" s="11" t="inlineStr">
+      <c r="M35" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M35" s="8" t="inlineStr">
+      <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N35" s="11" t="inlineStr">
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P35" s="12" t="inlineStr">
         <is>
           <t>All 6-operator fiber junction points on map.</t>
         </is>
@@ -2330,7 +2594,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="72" customHeight="1">
+    <row r="37" ht="80" customHeight="1">
       <c r="A37" s="5" t="n">
         <v>22</v>
       </c>
@@ -2361,15 +2625,20 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
+          <t>Bangladesh Railway</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
           <t>353</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>8 Core
 16 Core
@@ -2379,103 +2648,118 @@
 96 Core</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>Station Name A, Station Name B, Length (km), Total Core, Used Core, Unused Core</t>
         </is>
       </c>
-      <c r="K37" s="7" t="inlineStr">
+      <c r="L37" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L37" s="7" t="inlineStr">
+      <c r="M37" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M37" s="8" t="inlineStr">
+      <c r="N37" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N37" s="7" t="inlineStr">
-        <is>
-          <t>All 353 fiber route segments on map. Note: duplicate copy of same file exists in Railway folder — not used.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="72" customHeight="1">
-      <c r="A38" s="9" t="n">
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P37" s="7" t="inlineStr">
+        <is>
+          <t>All 353 fiber route segments on map. Duplicate copy of same file exists in Railway folder — not used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="80" customHeight="1">
+      <c r="A38" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Bangladesh Railway (BR)</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>Fiber Station Nodes</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>(Derived from railway Excel)</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F38" s="11" t="inlineStr">
+      <c r="F38" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Bangladesh Railway</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
         <is>
           <t>354</t>
         </is>
       </c>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="I38" s="12" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I38" s="11" t="inlineStr">
+      <c r="J38" s="12" t="inlineStr">
         <is>
           <t>Station junction nodes</t>
         </is>
       </c>
-      <c r="J38" s="11" t="inlineStr">
+      <c r="K38" s="12" t="inlineStr">
         <is>
           <t>Station name</t>
         </is>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="L38" s="12" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L38" s="11" t="inlineStr">
+      <c r="M38" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M38" s="8" t="inlineStr">
+      <c r="N38" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N38" s="11" t="inlineStr">
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P38" s="12" t="inlineStr">
         <is>
           <t>All 354 station nodes on map.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="72" customHeight="1">
+    <row r="39" ht="80" customHeight="1">
       <c r="A39" s="5" t="n">
         <v>24</v>
       </c>
@@ -2507,40 +2791,50 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
+          <t>Bangladesh Railway</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
           <t>2,675</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>Railway route segments</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>Route geometry</t>
         </is>
       </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr">
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="M39" s="8" t="inlineStr">
+      <c r="N39" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N39" s="7" t="inlineStr">
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>No gap — all records implemented.</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>Base railway track layer on map.</t>
         </is>
@@ -2553,7 +2847,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="72" customHeight="1">
+    <row r="41" ht="80" customHeight="1">
       <c r="A41" s="5" t="n">
         <v>25</v>
       </c>
@@ -2580,20 +2874,25 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>2020–2021</t>
+          <t>2020-2021</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
+          <t>BTRC / All ISPs</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
           <t>3,930</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="I41" s="7" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>Category-A ISPs
 Category-B ISPs
@@ -2601,81 +2900,87 @@
 (covers all districts nationwide)</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr">
+      <c r="K41" s="7" t="inlineStr">
         <is>
           <t>GID, POP Code, POP Name, POP Address, POP Capacity, ISP Name, Type of ISP, Lat, Lon, District, Division, Upazila, Union, Mouza</t>
         </is>
       </c>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="L41" s="7" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr">
-        <is>
-          <t>2020–2021</t>
-        </is>
-      </c>
-      <c r="M41" s="13" t="inlineStr">
+      <c r="M41" s="7" t="inlineStr">
+        <is>
+          <t>2020-2021</t>
+        </is>
+      </c>
+      <c r="N41" s="16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="N41" s="7" t="inlineStr">
-        <is>
-          <t>Data available and ready. Not yet implemented on map. Priority: High — add ISP POP overlay with category filter.</t>
+      <c r="O41" s="15" t="inlineStr">
+        <is>
+          <t>3,930 records not yet on map (100% gap).
+Data is fully available and ready for implementation.</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>High priority. Add ISP POP overlay with category filter (A/B/C) and district filter. Popup should show ISP name, capacity, address, admin.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ■  Yes — fully implemented on the map</t>
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Yes — fully implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ■  Partial — only a subset is on the map</t>
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Partial — only a subset is on the map</t>
         </is>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ■  No — data not yet implemented on the map</t>
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  No — data not yet implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ■  Indirect — used as a source for another file</t>
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Indirect — used as a source for another file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N4"/>
+  <autoFilter ref="A4:P4"/>
   <mergeCells count="18">
-    <mergeCell ref="A40:N40"/>
-    <mergeCell ref="A9:N9"/>
-    <mergeCell ref="A18:N18"/>
-    <mergeCell ref="A31:N31"/>
-    <mergeCell ref="A45:N45"/>
-    <mergeCell ref="A28:N28"/>
-    <mergeCell ref="A21:N21"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A36:N36"/>
-    <mergeCell ref="A7:N7"/>
-    <mergeCell ref="A25:N25"/>
-    <mergeCell ref="A43:N43"/>
-    <mergeCell ref="A33:N33"/>
-    <mergeCell ref="A5:N5"/>
-    <mergeCell ref="A46:N46"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A44:N44"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A28:P28"/>
+    <mergeCell ref="A46:P46"/>
+    <mergeCell ref="A13:P13"/>
+    <mergeCell ref="A33:P33"/>
+    <mergeCell ref="A36:P36"/>
+    <mergeCell ref="A44:P44"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A40:P40"/>
+    <mergeCell ref="A9:P9"/>
+    <mergeCell ref="A18:P18"/>
+    <mergeCell ref="A31:P31"/>
+    <mergeCell ref="A45:P45"/>
+    <mergeCell ref="A21:P21"/>
+    <mergeCell ref="A7:P7"/>
+    <mergeCell ref="A25:P25"/>
+    <mergeCell ref="A43:P43"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
feat: add master data inventory Excel (single consolidated sheet)
Updated BTRC_Master_Data_Inventory.xlsx to 19 columns:
- Dashboard Label / Button: exact UI toggle label in MapLayersPanel
- File Timestamp: source file last-modified datetime from disk
- Version / Git Commit: short hash + date from git log per data file
- Gap Analysis column with green/amber/red colour coding

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MapData/BTRC_Master_Data_Inventory.xlsx
+++ b/MapData/BTRC_Master_Data_Inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Data Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Data Inventory'!$A$4:$P$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Data Inventory'!$A$4:$S$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Master Data Inventory'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00166534"/>
       <sz val="9"/>
@@ -93,6 +99,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00991B1B"/>
       <sz val="9"/>
     </font>
@@ -196,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -219,10 +230,13 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -234,28 +248,34 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -623,43 +643,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="38" customWidth="1" min="18" max="18"/>
+    <col width="38" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BTRC IMS — Master Data Inventory  |  Submitted to BTRC for Validation</t>
+          <t>BTRC IMS -- Master Data Inventory  |  Submitted to BTRC for Validation</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per dataset. Covers: received file details, source, data types, usage status, gap analysis, and remarks.</t>
+          <t>One row per dataset. Covers: received file details, source, data types, dashboard mapping, file version, usage status, gap analysis, and remarks.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="4" customHeight="1"/>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>S/N</t>
@@ -727,15 +750,30 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
+          <t>Dashboard Label / Button</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>File Timestamp</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Version / Git Commit</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
           <t>Used on Map?</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Gap Analysis</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Notes / Remarks</t>
         </is>
@@ -815,15 +853,30 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
+          <t>Grameenphone &gt; Sites</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:46</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>d6971ec  2026-05-17</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P6" s="7" t="inlineStr">
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
         <is>
           <t>Admin (Division / District / Upazila) enriched via point-in-polygon lookup. 246 border-edge sites show '--' for admin fields.</t>
         </is>
@@ -904,17 +957,32 @@
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
+          <t>Robi &gt; Sites</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:46</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>4ea34be  2026-05-17</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O8" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P8" s="7" t="inlineStr">
-        <is>
-          <t>Three-category backhaul classification applied. Admin enriched via PIP. 169 border-edge sites show '--'.</t>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>Three-category backhaul classification (MW / Fiber / Both) applied. Admin enriched via PIP. 169 border-edge sites show '--'.</t>
         </is>
       </c>
     </row>
@@ -936,7 +1004,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>BTS Sites — Latest</t>
+          <t>BTS Sites -- Latest</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -993,97 +1061,127 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
+          <t>Banglalink &gt; BTS Sites (Latest)</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:46</t>
+        </is>
+      </c>
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>a98fd86  2026-05-17</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O10" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S10" s="7" t="inlineStr">
         <is>
           <t>Admin data taken directly from Excel (no PIP needed). Address field included in popup.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Banglalink</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>BTS Towers — Historical</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>BTS Towers -- Historical</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>3gtower.geojson</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Banglalink</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>13,208</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>4G sites
 3G only
 2G only</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>Site Code, Site Name, Generation (2G/3G/4G), Division, District, Upazila, Union, Vendor</t>
         </is>
       </c>
-      <c r="L11" s="12" t="inlineStr">
+      <c r="L11" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="M11" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N11" s="8" t="inlineStr">
+      <c r="N11" s="14" t="inlineStr">
+        <is>
+          <t>Banglalink &gt; Towers</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-04 18:35</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O11" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P11" s="12" t="inlineStr">
+      <c r="R11" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S11" s="13" t="inlineStr">
         <is>
           <t>Historical tower dataset. Filterable by generation on map.</t>
         </is>
@@ -1100,7 +1198,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Fiber Lines — Historical</t>
+          <t>Fiber Lines -- Historical</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1157,15 +1255,30 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
+          <t>Banglalink &gt; Fiber Lines</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-04 19:05</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O12" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P12" s="7" t="inlineStr">
+      <c r="R12" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
         <is>
           <t>Historical fiber route lines. Filterable by core count on map.</t>
         </is>
@@ -1189,7 +1302,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Network Points — Latest</t>
+          <t>Network Points -- Latest</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1250,65 +1363,80 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
+          <t>BTCL &gt; Points (Excel 2025)</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:45</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr">
-        <is>
-          <t>69 records removed (0.3% of total). Coordinates fell outside Bangladesh boundary — likely data-entry errors.</t>
-        </is>
-      </c>
-      <c r="P14" s="7" t="inlineStr">
-        <is>
-          <t>24,073 of 24,142 on map. Filtered points near borders should be verified and resubmitted by BTCL with corrected coordinates.</t>
+      <c r="R14" s="15" t="inlineStr">
+        <is>
+          <t>69 records removed (0.3% of total). Coordinates fell outside Bangladesh boundary -- likely data-entry errors.</t>
+        </is>
+      </c>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>24,073 of 24,142 on map. Filtered points should be verified and resubmitted by BTCL with corrected coordinates.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Fiber Lines — Historical</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Fiber Lines -- Historical</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>btcl-nttn-line.geojson</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>584</t>
         </is>
       </c>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr">
         <is>
           <t>MultiLineString</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>144+ Core
 96 Core
@@ -1317,32 +1445,47 @@
 &lt;24 Core</t>
         </is>
       </c>
-      <c r="K15" s="12" t="inlineStr">
+      <c r="K15" s="13" t="inlineStr">
         <is>
           <t>Operator Name, Line Name, Line Type, Core Count, Route Length (km), Cable Length (km), Duct Info, Division / District / Upazila</t>
         </is>
       </c>
-      <c r="L15" s="12" t="inlineStr">
+      <c r="L15" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="M15" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N15" s="8" t="inlineStr">
+      <c r="N15" s="14" t="inlineStr">
+        <is>
+          <t>BTCL-OLD &gt; Fiber Lines</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-05 14:00</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P15" s="12" t="inlineStr">
+      <c r="R15" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S15" s="13" t="inlineStr">
         <is>
           <t>All lines on map. Filterable by core-count band.</t>
         </is>
@@ -1359,7 +1502,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Network Nodes — Historical</t>
+          <t>Network Nodes -- Historical</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -1417,95 +1560,125 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
+          <t>BTCL-OLD &gt; Nodes</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:43</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O16" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P16" s="7" t="inlineStr">
+      <c r="R16" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S16" s="7" t="inlineStr">
         <is>
           <t>All nodes on map. Filterable by node type.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="80" customHeight="1">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>Union Project Locations</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>btcl-union-project-location.geojson</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>966</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J17" s="12" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>Union-level project markers</t>
         </is>
       </c>
-      <c r="K17" s="12" t="inlineStr">
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t>Location coordinates</t>
         </is>
       </c>
-      <c r="L17" s="12" t="inlineStr">
+      <c r="L17" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M17" s="12" t="inlineStr">
+      <c r="M17" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N17" s="8" t="inlineStr">
+      <c r="N17" s="14" t="inlineStr">
+        <is>
+          <t>BTCL-OLD &gt; Union Projects</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-05 12:41</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>1f15920  2026-05-05</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P17" s="12" t="inlineStr">
+      <c r="R17" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S17" s="13" t="inlineStr">
         <is>
           <t>All union project markers on map.</t>
         </is>
@@ -1585,70 +1758,85 @@
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="N19" s="14" t="inlineStr">
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>Fiber@Home &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-30 19:18</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q19" s="16" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="O19" s="15" t="inlineStr">
+      <c r="R19" s="17" t="inlineStr">
         <is>
           <t>123,162 lines not yet on map (87% gap).
 Currently showing: 18,405 of 141,567.
-Missing: full Aerial set (85k), full Burial set (53k), all OPGW (2,331).</t>
-        </is>
-      </c>
-      <c r="P19" s="7" t="inlineStr">
+Missing: full Aerial (85k), full Burial (53k), all OPGW (2,331).</t>
+        </is>
+      </c>
+      <c r="S19" s="7" t="inlineStr">
         <is>
           <t>Full re-ingestion from FHLFONLineExcel.xlsx required. Current map uses only a pre-converted subset.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Fiber@Home (FHLFON)</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>FHLFONPoint.shp + FHLFONPointExcel.xlsx
 (10 files: 8 shapefile + 1 Excel + 1 duplicate)</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Shapefile + XLSX</t>
         </is>
       </c>
-      <c r="F20" s="12" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="G20" s="12" t="inlineStr">
+      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Fiber@Home / FHLFON</t>
         </is>
       </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="H20" s="13" t="inlineStr">
         <is>
           <t>122,150</t>
         </is>
       </c>
-      <c r="I20" s="12" t="inlineStr">
+      <c r="I20" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J20" s="12" t="inlineStr">
+      <c r="J20" s="13" t="inlineStr">
         <is>
           <t>JE (Joint Enclosure): 38,097
 EP (End Point): 25,804
@@ -1667,34 +1855,49 @@
 Other / Noise: ~44</t>
         </is>
       </c>
-      <c r="K20" s="12" t="inlineStr">
+      <c r="K20" s="13" t="inlineStr">
         <is>
           <t>Year, Month, Operator Code, Operator Name, Point ID, Point Type, Point Name, Address, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="L20" s="12" t="inlineStr">
+      <c r="L20" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M20" s="12" t="inlineStr">
+      <c r="M20" s="13" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
       <c r="N20" s="14" t="inlineStr">
         <is>
+          <t>Fiber@Home &gt; Points</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:16</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q20" s="16" t="inlineStr">
+        <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="O20" s="15" t="inlineStr">
+      <c r="R20" s="17" t="inlineStr">
         <is>
           <t>27,197 points not on map (22% gap).
 Currently showing: 94,953 of 122,150.
 Missing types: Coupler (22,435), FL (16,558), BDB (1,390), Pole (479), LDP (387), PIT (26), Customer (25).</t>
         </is>
       </c>
-      <c r="P20" s="12" t="inlineStr">
+      <c r="S20" s="13" t="inlineStr">
         <is>
           <t>'Copy of FHLFONPointExcel.xlsx' is an exact duplicate and not used.</t>
         </is>
@@ -1776,70 +1979,85 @@
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="N22" s="14" t="inlineStr">
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>Summit &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-13 13:10</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q22" s="16" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="O22" s="15" t="inlineStr">
+      <c r="R22" s="17" t="inlineStr">
         <is>
           <t>79,357 lines not on map (77% gap).
 Currently showing: 23,157 of 102,514.
 Missing: majority of Aerial (78k) and Burial (22k) lines.</t>
         </is>
       </c>
-      <c r="P22" s="7" t="inlineStr">
+      <c r="S22" s="7" t="inlineStr">
         <is>
           <t>Full re-ingestion from Line_data.xlsx required. Current map uses a simplified 3-tier classification only.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="80" customHeight="1">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Summit Communications</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Point_data.xlsx + Point_data.shp
 (1 Excel + multiple shapefile components)</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>XLSX + Shapefile</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G23" s="13" t="inlineStr">
         <is>
           <t>Summit Communications</t>
         </is>
       </c>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr">
         <is>
           <t>68,850</t>
         </is>
       </c>
-      <c r="I23" s="12" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J23" s="12" t="inlineStr">
+      <c r="J23" s="13" t="inlineStr">
         <is>
           <t>TJB (Joint Box): 37,909
 HH (Hand Hole): 9,506
@@ -1858,34 +2076,49 @@
 Other: ~183</t>
         </is>
       </c>
-      <c r="K23" s="12" t="inlineStr">
+      <c r="K23" s="13" t="inlineStr">
         <is>
           <t>FID, Point ID, Year, Month, Operator Code, Operator Name, Point Type, Point Name, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="L23" s="12" t="inlineStr">
+      <c r="L23" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M23" s="12" t="inlineStr">
+      <c r="M23" s="13" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
       <c r="N23" s="14" t="inlineStr">
         <is>
+          <t>Summit &gt; Nodes + BTS</t>
+        </is>
+      </c>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>2026-04-13 13:12</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q23" s="16" t="inlineStr">
+        <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="O23" s="15" t="inlineStr">
+      <c r="R23" s="17" t="inlineStr">
         <is>
           <t>54,288 points not on map (79% gap).
 Currently showing: 14,562 of 68,850.
 Missing: TJB (37,909), EP (6,872), ODB (1,193), Node/TT (812), POP (666), POC (453), BS (422), Node/CBD (245), COLO/PoP (128), FAT (89), FDT (62).</t>
         </is>
       </c>
-      <c r="P23" s="12" t="inlineStr">
+      <c r="S23" s="13" t="inlineStr">
         <is>
           <t>Only Nodes (5,949) and BTS (8,613) currently on map.</t>
         </is>
@@ -1902,7 +2135,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Summit.rar (Archive — not extracted)</t>
+          <t>Summit.rar (Archive -- not extracted)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1937,7 +2170,7 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Unknown — archive not extracted</t>
+          <t>Unknown -- archive not extracted</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
@@ -1955,19 +2188,34 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="N24" s="16" t="inlineStr">
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>-- Not on map --</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="P24" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q24" s="18" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O24" s="13" t="inlineStr">
+      <c r="R24" s="15" t="inlineStr">
         <is>
           <t>Not yet extracted. Content and size unknown.</t>
         </is>
       </c>
-      <c r="P24" s="7" t="inlineStr">
-        <is>
-          <t>Archive file found in Railway folder. Must be extracted and analysed to determine if it contains additional network data.</t>
+      <c r="S24" s="7" t="inlineStr">
+        <is>
+          <t>Archive file in Railway folder. Must be extracted and analysed to check for additional network data.</t>
         </is>
       </c>
     </row>
@@ -2047,95 +2295,125 @@
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
+          <t>Bahon &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:16</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q26" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O26" s="15" t="inlineStr">
-        <is>
-          <t>No significant gap detected. Exact source count unverified (shapefile only — no Excel counterpart for cross-check).</t>
-        </is>
-      </c>
-      <c r="P26" s="7" t="inlineStr">
+      <c r="R26" s="17" t="inlineStr">
+        <is>
+          <t>No significant gap detected. Exact source count unverified (shapefile only -- no Excel counterpart for cross-check).</t>
+        </is>
+      </c>
+      <c r="S26" s="7" t="inlineStr">
         <is>
           <t>No Excel submission received from Bahon. Request Excel tabular data for BTRC records.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="80" customHeight="1">
-      <c r="A27" s="10" t="n">
+      <c r="A27" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Bahon Limited</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>(Derived from shapefile dataset)</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E27" s="13" t="inlineStr">
         <is>
           <t>Shapefile</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G27" s="12" t="inlineStr">
+      <c r="G27" s="13" t="inlineStr">
         <is>
           <t>Bahon Limited</t>
         </is>
       </c>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="H27" s="13" t="inlineStr">
         <is>
           <t>12,817</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J27" s="12" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>Network junction nodes</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr">
+      <c r="K27" s="13" t="inlineStr">
         <is>
           <t>Node coordinates</t>
         </is>
       </c>
-      <c r="L27" s="12" t="inlineStr">
+      <c r="L27" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M27" s="12" t="inlineStr">
+      <c r="M27" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N27" s="8" t="inlineStr">
+      <c r="N27" s="14" t="inlineStr">
+        <is>
+          <t>Bahon &gt; Nodes</t>
+        </is>
+      </c>
+      <c r="O27" s="13" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:16</t>
+        </is>
+      </c>
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q27" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O27" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P27" s="12" t="inlineStr">
+      <c r="R27" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S27" s="13" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -2165,7 +2443,7 @@
       <c r="D29" s="7" t="inlineStr">
         <is>
           <t>doc.kml
-(icon assets: mysavedplaces_closed.png, mysavedplaces_open.png)</t>
+(+ icon assets: mysavedplaces_closed.png, mysavedplaces_open.png)</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2220,95 +2498,125 @@
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
+          <t>InfoSarkar-3 &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:16</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O29" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P29" s="7" t="inlineStr">
+      <c r="R29" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S29" s="7" t="inlineStr">
         <is>
           <t>All lines on map with core-count filter.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="80" customHeight="1">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>InfoSarkar-3 (IS3)</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>doc.kml (same file)</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="13" t="inlineStr">
         <is>
           <t>KML</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="G30" s="13" t="inlineStr">
         <is>
           <t>InfoSarkar-3 / FHL</t>
         </is>
       </c>
-      <c r="H30" s="12" t="inlineStr">
+      <c r="H30" s="13" t="inlineStr">
         <is>
           <t>477</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr">
+      <c r="I30" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J30" s="12" t="inlineStr">
+      <c r="J30" s="13" t="inlineStr">
         <is>
           <t>Network junction nodes</t>
         </is>
       </c>
-      <c r="K30" s="12" t="inlineStr">
+      <c r="K30" s="13" t="inlineStr">
         <is>
           <t>Node coordinates</t>
         </is>
       </c>
-      <c r="L30" s="12" t="inlineStr">
+      <c r="L30" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M30" s="12" t="inlineStr">
+      <c r="M30" s="13" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N30" s="8" t="inlineStr">
+      <c r="N30" s="14" t="inlineStr">
+        <is>
+          <t>InfoSarkar-3 &gt; Nodes</t>
+        </is>
+      </c>
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:16</t>
+        </is>
+      </c>
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t>f903a24  2026-04-30</t>
+        </is>
+      </c>
+      <c r="Q30" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O30" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P30" s="12" t="inlineStr">
+      <c r="R30" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S30" s="13" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -2391,15 +2699,30 @@
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
+          <t>PGCB &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O32" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28 18:11</t>
+        </is>
+      </c>
+      <c r="P32" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q32" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O32" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P32" s="7" t="inlineStr">
+      <c r="R32" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S32" s="7" t="inlineStr">
         <is>
           <t>All OPGW lines on map. Filterable by voltage / line type.</t>
         </is>
@@ -2425,7 +2748,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Fiber Network — Lines</t>
+          <t>Fiber Network -- Lines</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -2486,66 +2809,81 @@
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
+          <t>Fiber Network &gt; Lines</t>
+        </is>
+      </c>
+      <c r="O34" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:46</t>
+        </is>
+      </c>
+      <c r="P34" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q34" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O34" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P34" s="7" t="inlineStr">
+      <c r="R34" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S34" s="7" t="inlineStr">
         <is>
           <t>All 6-operator inter-district fiber lines on map with operator colour filter.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="80" customHeight="1">
-      <c r="A35" s="10" t="n">
+      <c r="A35" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Multi-operator
 (GP, Robi, BTCL, BL, MOTN, BSCCL)</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>Fiber Network — Points</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Fiber Network -- Points</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>fiber_network_multiple_district.kmz (same file)</t>
         </is>
       </c>
-      <c r="E35" s="12" t="inlineStr">
+      <c r="E35" s="13" t="inlineStr">
         <is>
           <t>KMZ</t>
         </is>
       </c>
-      <c r="F35" s="12" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G35" s="12" t="inlineStr">
+      <c r="G35" s="13" t="inlineStr">
         <is>
           <t>BTRC / Multiple Operators</t>
         </is>
       </c>
-      <c r="H35" s="12" t="inlineStr">
+      <c r="H35" s="13" t="inlineStr">
         <is>
           <t>19,096</t>
         </is>
       </c>
-      <c r="I35" s="12" t="inlineStr">
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J35" s="12" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Grameenphone
 Robi
@@ -2556,32 +2894,47 @@
 Unknown</t>
         </is>
       </c>
-      <c r="K35" s="12" t="inlineStr">
+      <c r="K35" s="13" t="inlineStr">
         <is>
           <t>Name, Operator</t>
         </is>
       </c>
-      <c r="L35" s="12" t="inlineStr">
+      <c r="L35" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M35" s="12" t="inlineStr">
+      <c r="M35" s="13" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="N35" s="8" t="inlineStr">
+      <c r="N35" s="14" t="inlineStr">
+        <is>
+          <t>Fiber Network &gt; Points</t>
+        </is>
+      </c>
+      <c r="O35" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:46</t>
+        </is>
+      </c>
+      <c r="P35" s="13" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q35" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O35" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P35" s="12" t="inlineStr">
+      <c r="R35" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S35" s="13" t="inlineStr">
         <is>
           <t>All 6-operator fiber junction points on map.</t>
         </is>
@@ -2665,95 +3018,125 @@
       </c>
       <c r="N37" s="8" t="inlineStr">
         <is>
+          <t>Railway &gt; BR Fiber Lines</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:45</t>
+        </is>
+      </c>
+      <c r="P37" s="7" t="inlineStr">
+        <is>
+          <t>1f15920  2026-05-05</t>
+        </is>
+      </c>
+      <c r="Q37" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O37" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P37" s="7" t="inlineStr">
-        <is>
-          <t>All 353 fiber route segments on map. Duplicate copy of same file exists in Railway folder — not used.</t>
+      <c r="R37" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>All 353 fiber route segments on map. Duplicate copy in Railway folder -- not used.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="80" customHeight="1">
-      <c r="A38" s="10" t="n">
+      <c r="A38" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Bangladesh Railway (BR)</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>Fiber Station Nodes</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>(Derived from railway Excel)</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="13" t="inlineStr">
         <is>
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F38" s="12" t="inlineStr">
+      <c r="F38" s="13" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="G38" s="13" t="inlineStr">
         <is>
           <t>Bangladesh Railway</t>
         </is>
       </c>
-      <c r="H38" s="12" t="inlineStr">
+      <c r="H38" s="13" t="inlineStr">
         <is>
           <t>354</t>
         </is>
       </c>
-      <c r="I38" s="12" t="inlineStr">
+      <c r="I38" s="13" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J38" s="12" t="inlineStr">
+      <c r="J38" s="13" t="inlineStr">
         <is>
           <t>Station junction nodes</t>
         </is>
       </c>
-      <c r="K38" s="12" t="inlineStr">
+      <c r="K38" s="13" t="inlineStr">
         <is>
           <t>Station name</t>
         </is>
       </c>
-      <c r="L38" s="12" t="inlineStr">
+      <c r="L38" s="13" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M38" s="12" t="inlineStr">
+      <c r="M38" s="13" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="N38" s="8" t="inlineStr">
+      <c r="N38" s="14" t="inlineStr">
+        <is>
+          <t>Railway &gt; BR Fiber Nodes</t>
+        </is>
+      </c>
+      <c r="O38" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:45</t>
+        </is>
+      </c>
+      <c r="P38" s="13" t="inlineStr">
+        <is>
+          <t>1f15920  2026-05-05</t>
+        </is>
+      </c>
+      <c r="Q38" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O38" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P38" s="12" t="inlineStr">
+      <c r="R38" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S38" s="13" t="inlineStr">
         <is>
           <t>All 354 station nodes on map.</t>
         </is>
@@ -2826,15 +3209,30 @@
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
+          <t>Railway &gt; Railline</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-04 12:38</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O39" s="9" t="inlineStr">
-        <is>
-          <t>No gap — all records implemented.</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr">
+      <c r="R39" s="10" t="inlineStr">
+        <is>
+          <t>No gap -- all records implemented.</t>
+        </is>
+      </c>
+      <c r="S39" s="7" t="inlineStr">
         <is>
           <t>Base railway track layer on map.</t>
         </is>
@@ -2915,72 +3313,87 @@
           <t>2020-2021</t>
         </is>
       </c>
-      <c r="N41" s="16" t="inlineStr">
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>-- Not yet on map --</t>
+        </is>
+      </c>
+      <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-04 19:46</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="Q41" s="18" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O41" s="15" t="inlineStr">
+      <c r="R41" s="19" t="inlineStr">
         <is>
           <t>3,930 records not yet on map (100% gap).
 Data is fully available and ready for implementation.</t>
         </is>
       </c>
-      <c r="P41" s="7" t="inlineStr">
-        <is>
-          <t>High priority. Add ISP POP overlay with category filter (A/B/C) and district filter. Popup should show ISP name, capacity, address, admin.</t>
+      <c r="S41" s="7" t="inlineStr">
+        <is>
+          <t>High priority. Add ISP POP overlay with category filter (A/B/C) and district filter. Popup: ISP name, capacity, address, admin data.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [legend]  Yes — fully implemented on the map</t>
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Yes -- fully implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [legend]  Partial — only a subset is on the map</t>
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Partial -- only a subset is on the map</t>
         </is>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [legend]  No — data not yet implemented on the map</t>
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  No -- data not yet implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [legend]  Indirect — used as a source for another file</t>
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [legend]  Indirect -- used as a source for another file</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P4"/>
+  <autoFilter ref="A4:S4"/>
   <mergeCells count="18">
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A28:P28"/>
-    <mergeCell ref="A46:P46"/>
-    <mergeCell ref="A13:P13"/>
-    <mergeCell ref="A33:P33"/>
-    <mergeCell ref="A36:P36"/>
-    <mergeCell ref="A44:P44"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A40:P40"/>
-    <mergeCell ref="A9:P9"/>
-    <mergeCell ref="A18:P18"/>
-    <mergeCell ref="A31:P31"/>
-    <mergeCell ref="A45:P45"/>
-    <mergeCell ref="A21:P21"/>
-    <mergeCell ref="A7:P7"/>
-    <mergeCell ref="A25:P25"/>
-    <mergeCell ref="A43:P43"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A25:S25"/>
+    <mergeCell ref="A43:S43"/>
+    <mergeCell ref="A33:S33"/>
+    <mergeCell ref="A5:S5"/>
+    <mergeCell ref="A28:S28"/>
+    <mergeCell ref="A45:S45"/>
+    <mergeCell ref="A13:S13"/>
+    <mergeCell ref="A36:S36"/>
+    <mergeCell ref="A44:S44"/>
+    <mergeCell ref="A46:S46"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A40:S40"/>
+    <mergeCell ref="A9:S9"/>
+    <mergeCell ref="A18:S18"/>
+    <mergeCell ref="A31:S31"/>
+    <mergeCell ref="A21:S21"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A7:S7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
feat: replace git hash with human-readable Data Version column
Version column now shows 'v1 -- Dec 2025' style labels per dataset.
- v1 = initial load (current state)
- Increment to v2, v3 when operator resubmits updated data
- Readable by BTRC without any technical knowledge

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MapData/BTRC_Master_Data_Inventory.xlsx
+++ b/MapData/BTRC_Master_Data_Inventory.xlsx
@@ -661,7 +661,7 @@
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="38" customWidth="1" min="18" max="18"/>
     <col width="38" customWidth="1" min="19" max="19"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Version / Git Commit</t>
+          <t>Data Version</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>d6971ec  2026-05-17</t>
+          <t>v1 -- Dec 2025</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>4ea34be  2026-05-17</t>
+          <t>v1 -- Nov 2025</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>a98fd86  2026-05-17</t>
+          <t>v1 -- Dec 2025</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="P11" s="13" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q12" s="9" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- 2025</t>
         </is>
       </c>
       <c r="Q14" s="9" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q16" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="P17" s="13" t="inlineStr">
         <is>
-          <t>1f15920  2026-05-05</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Dec 2024</t>
         </is>
       </c>
       <c r="Q19" s="16" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="P20" s="13" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Dec 2024</t>
         </is>
       </c>
       <c r="Q20" s="16" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Mar 2026</t>
         </is>
       </c>
       <c r="Q22" s="16" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P23" s="13" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Mar 2026</t>
         </is>
       </c>
       <c r="Q23" s="16" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>-- Not processed --</t>
         </is>
       </c>
       <c r="Q24" s="18" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q26" s="9" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="P27" s="13" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="P30" s="13" t="inlineStr">
         <is>
-          <t>f903a24  2026-04-30</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q30" s="9" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q32" s="9" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- 2025</t>
         </is>
       </c>
       <c r="Q34" s="9" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="P35" s="13" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- 2025</t>
         </is>
       </c>
       <c r="Q35" s="9" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>1f15920  2026-05-05</t>
+          <t>v1 -- 2025</t>
         </is>
       </c>
       <c r="Q37" s="9" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="P38" s="13" t="inlineStr">
         <is>
-          <t>1f15920  2026-05-05</t>
+          <t>v1 -- 2025</t>
         </is>
       </c>
       <c r="Q38" s="9" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- Pre-2025</t>
         </is>
       </c>
       <c r="Q39" s="9" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>v1 -- 2020-2021</t>
         </is>
       </c>
       <c r="Q41" s="18" t="inlineStr">

</xml_diff>

<commit_message>
feat: derive Date Received and Data Version from actual file timestamps
Both columns now read the source file's mtime from disk:
- Date Received = file save date (e.g. 17 May 2026)
- Data Version  = v1 -- 17 May 2026 (auto-date, manual version number)
When an operator resubmits, replace the file and bump ver_num 1->2.
No hardcoded dates remain in the inventory script.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MapData/BTRC_Master_Data_Inventory.xlsx
+++ b/MapData/BTRC_Master_Data_Inventory.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,12 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
       <sz val="9"/>
     </font>
     <font>
@@ -114,7 +120,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +145,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -207,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -230,52 +241,55 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -651,7 +665,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
@@ -660,8 +674,8 @@
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="38" customWidth="1" min="18" max="18"/>
     <col width="38" customWidth="1" min="19" max="19"/>
@@ -677,7 +691,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per dataset. Covers: received file details, source, data types, dashboard mapping, file version, usage status, gap analysis, and remarks.</t>
+          <t>Date Received and Data Version are derived from actual file save dates on this machine. Version number increments each time an operator resubmits updated data.</t>
         </is>
       </c>
     </row>
@@ -810,9 +824,9 @@
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>18 Dec 2025</t>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -851,27 +865,27 @@
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>Grameenphone &gt; Sites</t>
         </is>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:46</t>
-        </is>
-      </c>
-      <c r="P6" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Dec 2025</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
+          <t>17 May 2026  12:46</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R6" s="10" t="inlineStr">
+      <c r="R6" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -913,9 +927,9 @@
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Nov 2025</t>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -955,27 +969,27 @@
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t>Robi &gt; Sites</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:46</t>
-        </is>
-      </c>
-      <c r="P8" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Nov 2025</t>
-        </is>
-      </c>
-      <c r="Q8" s="9" t="inlineStr">
+          <t>17 May 2026  12:46</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R8" s="10" t="inlineStr">
+      <c r="R8" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -1017,9 +1031,9 @@
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Dec 2025</t>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1059,27 +1073,27 @@
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="N10" s="8" t="inlineStr">
+      <c r="N10" s="9" t="inlineStr">
         <is>
           <t>Banglalink &gt; BTS Sites (Latest)</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:46</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Dec 2025</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
+          <t>17 May 2026  12:46</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R10" s="10" t="inlineStr">
+      <c r="R10" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -1091,97 +1105,97 @@
       </c>
     </row>
     <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Banglalink</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>BTS Towers -- Historical</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>3gtower.geojson</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>04 May 2026</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>Banglalink</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>13,208</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>4G sites
 3G only
 2G only</t>
         </is>
       </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="K11" s="14" t="inlineStr">
         <is>
           <t>Site Code, Site Name, Generation (2G/3G/4G), Division, District, Upazila, Union, Vendor</t>
         </is>
       </c>
-      <c r="L11" s="13" t="inlineStr">
+      <c r="L11" s="14" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M11" s="13" t="inlineStr">
+      <c r="M11" s="14" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N11" s="14" t="inlineStr">
+      <c r="N11" s="15" t="inlineStr">
         <is>
           <t>Banglalink &gt; Towers</t>
         </is>
       </c>
-      <c r="O11" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-04 18:35</t>
-        </is>
-      </c>
-      <c r="P11" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="O11" s="14" t="inlineStr">
+        <is>
+          <t>04 May 2026  18:35</t>
+        </is>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 04 May 2026</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R11" s="10" t="inlineStr">
+      <c r="R11" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S11" s="13" t="inlineStr">
+      <c r="S11" s="14" t="inlineStr">
         <is>
           <t>Historical tower dataset. Filterable by generation on map.</t>
         </is>
@@ -1211,9 +1225,9 @@
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>04 May 2026</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1253,27 +1267,27 @@
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N12" s="8" t="inlineStr">
+      <c r="N12" s="9" t="inlineStr">
         <is>
           <t>Banglalink &gt; Fiber Lines</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>2026-05-04 19:05</t>
-        </is>
-      </c>
-      <c r="P12" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q12" s="9" t="inlineStr">
+          <t>04 May 2026  19:05</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 04 May 2026</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R12" s="10" t="inlineStr">
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -1315,9 +1329,9 @@
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1361,27 +1375,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="N14" s="9" t="inlineStr">
         <is>
           <t>BTCL &gt; Points (Excel 2025)</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:45</t>
-        </is>
-      </c>
-      <c r="P14" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- 2025</t>
-        </is>
-      </c>
-      <c r="Q14" s="9" t="inlineStr">
+          <t>17 May 2026  12:45</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R14" s="15" t="inlineStr">
+      <c r="R14" s="16" t="inlineStr">
         <is>
           <t>69 records removed (0.3% of total). Coordinates fell outside Bangladesh boundary -- likely data-entry errors.</t>
         </is>
@@ -1393,50 +1407,50 @@
       </c>
     </row>
     <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Fiber Lines -- Historical</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>btcl-nttn-line.geojson</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>05 May 2026</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>584</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>MultiLineString</t>
         </is>
       </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>144+ Core
 96 Core
@@ -1445,47 +1459,47 @@
 &lt;24 Core</t>
         </is>
       </c>
-      <c r="K15" s="13" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
         <is>
           <t>Operator Name, Line Name, Line Type, Core Count, Route Length (km), Cable Length (km), Duct Info, Division / District / Upazila</t>
         </is>
       </c>
-      <c r="L15" s="13" t="inlineStr">
+      <c r="L15" s="14" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M15" s="13" t="inlineStr">
+      <c r="M15" s="14" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N15" s="14" t="inlineStr">
+      <c r="N15" s="15" t="inlineStr">
         <is>
           <t>BTCL-OLD &gt; Fiber Lines</t>
         </is>
       </c>
-      <c r="O15" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-05 14:00</t>
-        </is>
-      </c>
-      <c r="P15" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="O15" s="14" t="inlineStr">
+        <is>
+          <t>05 May 2026  14:00</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 05 May 2026</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R15" s="10" t="inlineStr">
+      <c r="R15" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S15" s="13" t="inlineStr">
+      <c r="S15" s="14" t="inlineStr">
         <is>
           <t>All lines on map. Filterable by core-count band.</t>
         </is>
@@ -1515,9 +1529,9 @@
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>05 May 2026</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1558,27 +1572,27 @@
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N16" s="8" t="inlineStr">
+      <c r="N16" s="9" t="inlineStr">
         <is>
           <t>BTCL-OLD &gt; Nodes</t>
         </is>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>2026-05-05 12:43</t>
-        </is>
-      </c>
-      <c r="P16" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q16" s="9" t="inlineStr">
+          <t>05 May 2026  12:43</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 05 May 2026</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R16" s="10" t="inlineStr">
+      <c r="R16" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -1590,95 +1604,95 @@
       </c>
     </row>
     <row r="17" ht="80" customHeight="1">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>BTCL</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Union Project Locations</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>btcl-union-project-location.geojson</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>05 May 2026</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>BTCL</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>966</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>Union-level project markers</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Location coordinates</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>WGS84</t>
+        </is>
+      </c>
+      <c r="M17" s="14" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>BTCL</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>966</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="J17" s="13" t="inlineStr">
-        <is>
-          <t>Union-level project markers</t>
-        </is>
-      </c>
-      <c r="K17" s="13" t="inlineStr">
-        <is>
-          <t>Location coordinates</t>
-        </is>
-      </c>
-      <c r="L17" s="13" t="inlineStr">
-        <is>
-          <t>WGS84</t>
-        </is>
-      </c>
-      <c r="M17" s="13" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="N17" s="14" t="inlineStr">
+      <c r="N17" s="15" t="inlineStr">
         <is>
           <t>BTCL-OLD &gt; Union Projects</t>
         </is>
       </c>
-      <c r="O17" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-05 12:41</t>
-        </is>
-      </c>
-      <c r="P17" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="O17" s="14" t="inlineStr">
+        <is>
+          <t>05 May 2026  12:41</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 05 May 2026</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R17" s="10" t="inlineStr">
+      <c r="R17" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S17" s="13" t="inlineStr">
+      <c r="S17" s="14" t="inlineStr">
         <is>
           <t>All union project markers on map.</t>
         </is>
@@ -1716,9 +1730,9 @@
           <t>Shapefile + XLSX</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Dec 2024</t>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>30 Apr 2026</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1758,27 +1772,27 @@
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="N19" s="8" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr">
         <is>
           <t>Fiber@Home &gt; Lines</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>2026-04-30 19:18</t>
-        </is>
-      </c>
-      <c r="P19" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Dec 2024</t>
-        </is>
-      </c>
-      <c r="Q19" s="16" t="inlineStr">
+          <t>30 Apr 2026  19:18</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 30 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q19" s="17" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="R19" s="17" t="inlineStr">
+      <c r="R19" s="18" t="inlineStr">
         <is>
           <t>123,162 lines not yet on map (87% gap).
 Currently showing: 18,405 of 141,567.
@@ -1792,51 +1806,51 @@
       </c>
     </row>
     <row r="20" ht="80" customHeight="1">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Fiber@Home (FHLFON)</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>FHLFONPoint.shp + FHLFONPointExcel.xlsx
 (10 files: 8 shapefile + 1 Excel + 1 duplicate)</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Shapefile + XLSX</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>Dec 2024</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>Fiber@Home / FHLFON</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>122,150</t>
         </is>
       </c>
-      <c r="I20" s="13" t="inlineStr">
+      <c r="I20" s="14" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>JE (Joint Enclosure): 38,097
 EP (End Point): 25,804
@@ -1855,49 +1869,49 @@
 Other / Noise: ~44</t>
         </is>
       </c>
-      <c r="K20" s="13" t="inlineStr">
+      <c r="K20" s="14" t="inlineStr">
         <is>
           <t>Year, Month, Operator Code, Operator Name, Point ID, Point Type, Point Name, Address, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="L20" s="13" t="inlineStr">
+      <c r="L20" s="14" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M20" s="13" t="inlineStr">
+      <c r="M20" s="14" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="N20" s="14" t="inlineStr">
+      <c r="N20" s="15" t="inlineStr">
         <is>
           <t>Fiber@Home &gt; Points</t>
         </is>
       </c>
-      <c r="O20" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-28 18:16</t>
-        </is>
-      </c>
-      <c r="P20" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Dec 2024</t>
-        </is>
-      </c>
-      <c r="Q20" s="16" t="inlineStr">
+      <c r="O20" s="14" t="inlineStr">
+        <is>
+          <t>28 Apr 2026  18:16</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q20" s="17" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="R20" s="17" t="inlineStr">
+      <c r="R20" s="18" t="inlineStr">
         <is>
           <t>27,197 points not on map (22% gap).
 Currently showing: 94,953 of 122,150.
 Missing types: Coupler (22,435), FL (16,558), BDB (1,390), Pole (479), LDP (387), PIT (26), Customer (25).</t>
         </is>
       </c>
-      <c r="S20" s="13" t="inlineStr">
+      <c r="S20" s="14" t="inlineStr">
         <is>
           <t>'Copy of FHLFONPointExcel.xlsx' is an exact duplicate and not used.</t>
         </is>
@@ -1935,9 +1949,9 @@
           <t>XLSX + Shapefile</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Mar 2026</t>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>13 Apr 2026</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1979,27 +1993,27 @@
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="N22" s="8" t="inlineStr">
+      <c r="N22" s="9" t="inlineStr">
         <is>
           <t>Summit &gt; Lines</t>
         </is>
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
-          <t>2026-04-13 13:10</t>
-        </is>
-      </c>
-      <c r="P22" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Mar 2026</t>
-        </is>
-      </c>
-      <c r="Q22" s="16" t="inlineStr">
+          <t>13 Apr 2026  13:10</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 13 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q22" s="17" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="R22" s="17" t="inlineStr">
+      <c r="R22" s="18" t="inlineStr">
         <is>
           <t>79,357 lines not on map (77% gap).
 Currently showing: 23,157 of 102,514.
@@ -2013,51 +2027,51 @@
       </c>
     </row>
     <row r="23" ht="80" customHeight="1">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Summit Communications</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Network Points</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Point_data.xlsx + Point_data.shp
 (1 Excel + multiple shapefile components)</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>XLSX + Shapefile</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Mar 2026</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>13 Apr 2026</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>Summit Communications</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>68,850</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr">
+      <c r="I23" s="14" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="J23" s="14" t="inlineStr">
         <is>
           <t>TJB (Joint Box): 37,909
 HH (Hand Hole): 9,506
@@ -2076,49 +2090,49 @@
 Other: ~183</t>
         </is>
       </c>
-      <c r="K23" s="13" t="inlineStr">
+      <c r="K23" s="14" t="inlineStr">
         <is>
           <t>FID, Point ID, Year, Month, Operator Code, Operator Name, Point Type, Point Name, Latitude, Longitude, Feature Code</t>
         </is>
       </c>
-      <c r="L23" s="13" t="inlineStr">
+      <c r="L23" s="14" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M23" s="13" t="inlineStr">
+      <c r="M23" s="14" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="N23" s="14" t="inlineStr">
+      <c r="N23" s="15" t="inlineStr">
         <is>
           <t>Summit &gt; Nodes + BTS</t>
         </is>
       </c>
-      <c r="O23" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-13 13:12</t>
-        </is>
-      </c>
-      <c r="P23" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Mar 2026</t>
-        </is>
-      </c>
-      <c r="Q23" s="16" t="inlineStr">
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>13 Apr 2026  13:12</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 13 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q23" s="17" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="R23" s="17" t="inlineStr">
+      <c r="R23" s="18" t="inlineStr">
         <is>
           <t>54,288 points not on map (79% gap).
 Currently showing: 14,562 of 68,850.
 Missing: TJB (37,909), EP (6,872), ODB (1,193), Node/TT (812), POP (666), POC (453), BS (422), Node/CBD (245), COLO/PoP (128), FAT (89), FDT (62).</t>
         </is>
       </c>
-      <c r="S23" s="13" t="inlineStr">
+      <c r="S23" s="14" t="inlineStr">
         <is>
           <t>Only Nodes (5,949) and BTS (8,613) currently on map.</t>
         </is>
@@ -2148,9 +2162,9 @@
           <t>RAR Archive</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Not specified</t>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>04 May 2026</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -2188,27 +2202,27 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="N24" s="8" t="inlineStr">
+      <c r="N24" s="9" t="inlineStr">
         <is>
           <t>-- Not on map --</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="P24" s="7" t="inlineStr">
-        <is>
-          <t>-- Not processed --</t>
-        </is>
-      </c>
-      <c r="Q24" s="18" t="inlineStr">
+          <t>04 May 2026  15:37</t>
+        </is>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 04 May 2026</t>
+        </is>
+      </c>
+      <c r="Q24" s="19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R24" s="15" t="inlineStr">
+      <c r="R24" s="16" t="inlineStr">
         <is>
           <t>Not yet extracted. Content and size unknown.</t>
         </is>
@@ -2251,9 +2265,9 @@
           <t>Shapefile</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -2293,27 +2307,27 @@
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N26" s="8" t="inlineStr">
+      <c r="N26" s="9" t="inlineStr">
         <is>
           <t>Bahon &gt; Lines</t>
         </is>
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
-          <t>2026-04-28 18:16</t>
-        </is>
-      </c>
-      <c r="P26" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q26" s="9" t="inlineStr">
+          <t>28 Apr 2026  18:16</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q26" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R26" s="17" t="inlineStr">
+      <c r="R26" s="18" t="inlineStr">
         <is>
           <t>No significant gap detected. Exact source count unverified (shapefile only -- no Excel counterpart for cross-check).</t>
         </is>
@@ -2325,95 +2339,95 @@
       </c>
     </row>
     <row r="27" ht="80" customHeight="1">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Bahon Limited</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>(Derived from shapefile dataset)</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Shapefile</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>Bahon Limited</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>12,817</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J27" s="14" t="inlineStr">
+        <is>
+          <t>Network junction nodes</t>
+        </is>
+      </c>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>Node coordinates</t>
+        </is>
+      </c>
+      <c r="L27" s="14" t="inlineStr">
+        <is>
+          <t>WGS84</t>
+        </is>
+      </c>
+      <c r="M27" s="14" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>Bahon Limited</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>12,817</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="J27" s="13" t="inlineStr">
-        <is>
-          <t>Network junction nodes</t>
-        </is>
-      </c>
-      <c r="K27" s="13" t="inlineStr">
-        <is>
-          <t>Node coordinates</t>
-        </is>
-      </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>WGS84</t>
-        </is>
-      </c>
-      <c r="M27" s="13" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="N27" s="14" t="inlineStr">
+      <c r="N27" s="15" t="inlineStr">
         <is>
           <t>Bahon &gt; Nodes</t>
         </is>
       </c>
-      <c r="O27" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-28 18:16</t>
-        </is>
-      </c>
-      <c r="P27" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q27" s="9" t="inlineStr">
+      <c r="O27" s="14" t="inlineStr">
+        <is>
+          <t>28 Apr 2026  18:16</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q27" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R27" s="10" t="inlineStr">
+      <c r="R27" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S27" s="13" t="inlineStr">
+      <c r="S27" s="14" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -2451,9 +2465,9 @@
           <t>KML</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -2496,27 +2510,27 @@
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N29" s="8" t="inlineStr">
+      <c r="N29" s="9" t="inlineStr">
         <is>
           <t>InfoSarkar-3 &gt; Lines</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
-          <t>2026-04-28 18:16</t>
-        </is>
-      </c>
-      <c r="P29" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q29" s="9" t="inlineStr">
+          <t>28 Apr 2026  18:16</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q29" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R29" s="10" t="inlineStr">
+      <c r="R29" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -2528,95 +2542,95 @@
       </c>
     </row>
     <row r="30" ht="80" customHeight="1">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>InfoSarkar-3 (IS3)</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>Network Nodes</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>doc.kml (same file)</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>KML</t>
         </is>
       </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>InfoSarkar-3 / FHL</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>477</t>
+        </is>
+      </c>
+      <c r="I30" s="14" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J30" s="14" t="inlineStr">
+        <is>
+          <t>Network junction nodes</t>
+        </is>
+      </c>
+      <c r="K30" s="14" t="inlineStr">
+        <is>
+          <t>Node coordinates</t>
+        </is>
+      </c>
+      <c r="L30" s="14" t="inlineStr">
+        <is>
+          <t>WGS84</t>
+        </is>
+      </c>
+      <c r="M30" s="14" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>InfoSarkar-3 / FHL</t>
-        </is>
-      </c>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>477</t>
-        </is>
-      </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>Network junction nodes</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>Node coordinates</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>WGS84</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="N30" s="14" t="inlineStr">
+      <c r="N30" s="15" t="inlineStr">
         <is>
           <t>InfoSarkar-3 &gt; Nodes</t>
         </is>
       </c>
-      <c r="O30" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-28 18:16</t>
-        </is>
-      </c>
-      <c r="P30" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q30" s="9" t="inlineStr">
+      <c r="O30" s="14" t="inlineStr">
+        <is>
+          <t>28 Apr 2026  18:16</t>
+        </is>
+      </c>
+      <c r="P30" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q30" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R30" s="10" t="inlineStr">
+      <c r="R30" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S30" s="13" t="inlineStr">
+      <c r="S30" s="14" t="inlineStr">
         <is>
           <t>All nodes on map.</t>
         </is>
@@ -2653,9 +2667,9 @@
           <t>KML</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>28 Apr 2026</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2697,27 +2711,27 @@
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="N32" s="8" t="inlineStr">
+      <c r="N32" s="9" t="inlineStr">
         <is>
           <t>PGCB &gt; Lines</t>
         </is>
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
-          <t>2026-04-28 18:11</t>
-        </is>
-      </c>
-      <c r="P32" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q32" s="9" t="inlineStr">
+          <t>28 Apr 2026  18:11</t>
+        </is>
+      </c>
+      <c r="P32" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 28 Apr 2026</t>
+        </is>
+      </c>
+      <c r="Q32" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R32" s="10" t="inlineStr">
+      <c r="R32" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -2761,9 +2775,9 @@
           <t>KMZ</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2807,27 +2821,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="N34" s="8" t="inlineStr">
+      <c r="N34" s="9" t="inlineStr">
         <is>
           <t>Fiber Network &gt; Lines</t>
         </is>
       </c>
       <c r="O34" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:46</t>
-        </is>
-      </c>
-      <c r="P34" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- 2025</t>
-        </is>
-      </c>
-      <c r="Q34" s="9" t="inlineStr">
+          <t>17 May 2026  12:46</t>
+        </is>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q34" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R34" s="10" t="inlineStr">
+      <c r="R34" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -2839,51 +2853,51 @@
       </c>
     </row>
     <row r="35" ht="80" customHeight="1">
-      <c r="A35" s="11" t="n">
+      <c r="A35" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Multi-operator
 (GP, Robi, BTCL, BL, MOTN, BSCCL)</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Fiber Network -- Points</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>fiber_network_multiple_district.kmz (same file)</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>KMZ</t>
         </is>
       </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>BTRC / Multiple Operators</t>
         </is>
       </c>
-      <c r="H35" s="13" t="inlineStr">
+      <c r="H35" s="14" t="inlineStr">
         <is>
           <t>19,096</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr">
+      <c r="I35" s="14" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J35" s="13" t="inlineStr">
+      <c r="J35" s="14" t="inlineStr">
         <is>
           <t>Grameenphone
 Robi
@@ -2894,47 +2908,47 @@
 Unknown</t>
         </is>
       </c>
-      <c r="K35" s="13" t="inlineStr">
+      <c r="K35" s="14" t="inlineStr">
         <is>
           <t>Name, Operator</t>
         </is>
       </c>
-      <c r="L35" s="13" t="inlineStr">
+      <c r="L35" s="14" t="inlineStr">
         <is>
           <t>WGS84</t>
         </is>
       </c>
-      <c r="M35" s="13" t="inlineStr">
+      <c r="M35" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="N35" s="14" t="inlineStr">
+      <c r="N35" s="15" t="inlineStr">
         <is>
           <t>Fiber Network &gt; Points</t>
         </is>
       </c>
-      <c r="O35" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-17 12:46</t>
-        </is>
-      </c>
-      <c r="P35" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- 2025</t>
-        </is>
-      </c>
-      <c r="Q35" s="9" t="inlineStr">
+      <c r="O35" s="14" t="inlineStr">
+        <is>
+          <t>17 May 2026  12:46</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q35" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R35" s="10" t="inlineStr">
+      <c r="R35" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S35" s="13" t="inlineStr">
+      <c r="S35" s="14" t="inlineStr">
         <is>
           <t>All 6-operator fiber junction points on map.</t>
         </is>
@@ -2971,9 +2985,9 @@
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -3016,27 +3030,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="N37" s="8" t="inlineStr">
+      <c r="N37" s="9" t="inlineStr">
         <is>
           <t>Railway &gt; BR Fiber Lines</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
         <is>
-          <t>2026-05-17 12:45</t>
-        </is>
-      </c>
-      <c r="P37" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- 2025</t>
-        </is>
-      </c>
-      <c r="Q37" s="9" t="inlineStr">
+          <t>17 May 2026  12:45</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q37" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R37" s="10" t="inlineStr">
+      <c r="R37" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -3048,95 +3062,95 @@
       </c>
     </row>
     <row r="38" ht="80" customHeight="1">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Bangladesh Railway (BR)</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Fiber Station Nodes</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>(Derived from railway Excel)</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>XLSX</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>Bangladesh Railway</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="I38" s="14" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J38" s="14" t="inlineStr">
+        <is>
+          <t>Station junction nodes</t>
+        </is>
+      </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>Station name</t>
+        </is>
+      </c>
+      <c r="L38" s="14" t="inlineStr">
+        <is>
+          <t>WGS84</t>
+        </is>
+      </c>
+      <c r="M38" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>Bangladesh Railway</t>
-        </is>
-      </c>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>354</t>
-        </is>
-      </c>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="J38" s="13" t="inlineStr">
-        <is>
-          <t>Station junction nodes</t>
-        </is>
-      </c>
-      <c r="K38" s="13" t="inlineStr">
-        <is>
-          <t>Station name</t>
-        </is>
-      </c>
-      <c r="L38" s="13" t="inlineStr">
-        <is>
-          <t>WGS84</t>
-        </is>
-      </c>
-      <c r="M38" s="13" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="N38" s="14" t="inlineStr">
+      <c r="N38" s="15" t="inlineStr">
         <is>
           <t>Railway &gt; BR Fiber Nodes</t>
         </is>
       </c>
-      <c r="O38" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-17 12:45</t>
-        </is>
-      </c>
-      <c r="P38" s="13" t="inlineStr">
-        <is>
-          <t>v1 -- 2025</t>
-        </is>
-      </c>
-      <c r="Q38" s="9" t="inlineStr">
+      <c r="O38" s="14" t="inlineStr">
+        <is>
+          <t>17 May 2026  12:45</t>
+        </is>
+      </c>
+      <c r="P38" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 17 May 2026</t>
+        </is>
+      </c>
+      <c r="Q38" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R38" s="10" t="inlineStr">
+      <c r="R38" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
       </c>
-      <c r="S38" s="13" t="inlineStr">
+      <c r="S38" s="14" t="inlineStr">
         <is>
           <t>All 354 station nodes on map.</t>
         </is>
@@ -3167,67 +3181,67 @@
           <t>GeoJSON + Shapefile</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>04 May 2026</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Bangladesh Railway</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>2,675</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>Railway route segments</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>Route geometry</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>WGS84</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>Pre-2025</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>Bangladesh Railway</t>
-        </is>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>2,675</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>LineString</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>Railway route segments</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>Route geometry</t>
-        </is>
-      </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>WGS84</t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>Pre-2025</t>
-        </is>
-      </c>
-      <c r="N39" s="8" t="inlineStr">
+      <c r="N39" s="9" t="inlineStr">
         <is>
           <t>Railway &gt; Railline</t>
         </is>
       </c>
       <c r="O39" s="7" t="inlineStr">
         <is>
-          <t>2026-05-04 12:38</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- Pre-2025</t>
-        </is>
-      </c>
-      <c r="Q39" s="9" t="inlineStr">
+          <t>04 May 2026  12:38</t>
+        </is>
+      </c>
+      <c r="P39" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 04 May 2026</t>
+        </is>
+      </c>
+      <c r="Q39" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="R39" s="10" t="inlineStr">
+      <c r="R39" s="11" t="inlineStr">
         <is>
           <t>No gap -- all records implemented.</t>
         </is>
@@ -3270,9 +3284,9 @@
           <t>GeoJSON + JSON</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>2020-2021</t>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>04 May 2026</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -3313,27 +3327,27 @@
           <t>2020-2021</t>
         </is>
       </c>
-      <c r="N41" s="8" t="inlineStr">
+      <c r="N41" s="9" t="inlineStr">
         <is>
           <t>-- Not yet on map --</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
         <is>
-          <t>2026-05-04 19:46</t>
-        </is>
-      </c>
-      <c r="P41" s="7" t="inlineStr">
-        <is>
-          <t>v1 -- 2020-2021</t>
-        </is>
-      </c>
-      <c r="Q41" s="18" t="inlineStr">
+          <t>04 May 2026  19:46</t>
+        </is>
+      </c>
+      <c r="P41" s="8" t="inlineStr">
+        <is>
+          <t>v1 -- 04 May 2026</t>
+        </is>
+      </c>
+      <c r="Q41" s="19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R41" s="19" t="inlineStr">
+      <c r="R41" s="20" t="inlineStr">
         <is>
           <t>3,930 records not yet on map (100% gap).
 Data is fully available and ready for implementation.</t>
@@ -3346,28 +3360,28 @@
       </c>
     </row>
     <row r="43" ht="14" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  [legend]  Yes -- fully implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="21" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">  [legend]  Partial -- only a subset is on the map</t>
         </is>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="A45" s="22" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  [legend]  No -- data not yet implemented on the map</t>
         </is>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  [legend]  Indirect -- used as a source for another file</t>
         </is>

</xml_diff>